<commit_message>
Complete Sprint 5 cash flow intelligence, NLP, and reporting
</commit_message>
<xml_diff>
--- a/output/cashflow_intelligence.xlsx
+++ b/output/cashflow_intelligence.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K93"/>
+  <dimension ref="A1:L93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,6 +472,11 @@
           <t>capital_allocation_label</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>capital_allocation_pattern</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -517,6 +522,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -562,6 +572,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -607,6 +622,11 @@
           <t>Neutral</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -652,6 +672,11 @@
           <t>Neutral</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -697,6 +722,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -742,6 +772,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -787,6 +822,11 @@
           <t>Neutral</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -832,6 +872,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -877,6 +922,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -922,6 +972,11 @@
           <t>Distress Signal</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -967,6 +1022,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1012,6 +1072,11 @@
           <t>Distress Signal</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1057,6 +1122,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1102,6 +1172,11 @@
           <t>Distress Signal</t>
         </is>
       </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1147,6 +1222,11 @@
           <t>Distress Signal</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1192,6 +1272,11 @@
           <t>Neutral</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1237,6 +1322,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1282,6 +1372,11 @@
           <t>Distress Signal</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1327,6 +1422,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1372,6 +1472,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1417,6 +1522,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1462,6 +1572,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1507,6 +1622,11 @@
           <t>Distress Signal</t>
         </is>
       </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1552,6 +1672,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1597,6 +1722,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1642,6 +1772,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1687,6 +1822,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1732,6 +1872,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1777,6 +1922,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1822,6 +1972,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1867,6 +2022,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1912,6 +2072,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1957,6 +2122,11 @@
           <t>Neutral</t>
         </is>
       </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2002,6 +2172,11 @@
           <t>Distress Signal</t>
         </is>
       </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2047,6 +2222,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2092,6 +2272,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2137,6 +2322,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2182,6 +2372,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2227,6 +2422,11 @@
           <t>Neutral</t>
         </is>
       </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2272,6 +2472,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2317,6 +2522,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2362,6 +2572,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2407,6 +2622,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2452,6 +2672,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2497,6 +2722,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2542,6 +2772,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2587,6 +2822,11 @@
           <t>Neutral</t>
         </is>
       </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Pre-Revenue</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2632,6 +2872,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2677,6 +2922,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2722,6 +2972,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2767,6 +3022,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2812,6 +3072,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2857,6 +3122,11 @@
           <t>Neutral</t>
         </is>
       </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2902,6 +3172,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2947,6 +3222,11 @@
           <t>Neutral</t>
         </is>
       </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2992,6 +3272,11 @@
           <t>Neutral</t>
         </is>
       </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3037,6 +3322,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3082,6 +3372,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3127,6 +3422,11 @@
           <t>Neutral</t>
         </is>
       </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3172,6 +3472,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3217,6 +3522,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3262,6 +3572,11 @@
           <t>Distress Signal</t>
         </is>
       </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3307,6 +3622,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3352,6 +3672,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3397,6 +3722,11 @@
           <t>Neutral</t>
         </is>
       </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3442,6 +3772,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3487,6 +3822,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3532,6 +3872,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3577,6 +3922,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3622,6 +3972,11 @@
           <t>Distress Signal</t>
         </is>
       </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3663,6 +4018,11 @@
         <v>1</v>
       </c>
       <c r="K72" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
         <is>
           <t>Reinvestor</t>
         </is>
@@ -3710,6 +4070,11 @@
           <t>Distress Signal</t>
         </is>
       </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3755,6 +4120,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3800,6 +4170,11 @@
           <t>Distress Signal</t>
         </is>
       </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3845,6 +4220,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3890,6 +4270,11 @@
           <t>Neutral</t>
         </is>
       </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3935,6 +4320,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3980,6 +4370,11 @@
           <t>Distress Signal</t>
         </is>
       </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4025,6 +4420,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4070,6 +4470,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4115,6 +4520,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4160,6 +4570,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4205,6 +4620,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4250,6 +4670,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4295,6 +4720,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4340,6 +4770,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4385,6 +4820,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4430,6 +4870,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4475,6 +4920,11 @@
           <t>Cash Generator</t>
         </is>
       </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4518,6 +4968,11 @@
       <c r="K91" t="inlineStr">
         <is>
           <t>Distress Signal</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
     </row>
@@ -4561,6 +5016,11 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4600,6 +5060,11 @@
       <c r="K93" t="inlineStr">
         <is>
           <t>Cash Generator</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>

</xml_diff>